<commit_message>
#7 eSpark BOM updated.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark-BOM.xlsx
+++ b/Deliverables/BOM/eSpark-BOM.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ezlo-thermostat\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ezlo-thermostat\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC290C2-1EFE-4481-B4C3-A422BC4FF394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="10 Boards" sheetId="1" r:id="rId1"/>
     <sheet name="1000 Boards" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="118">
   <si>
     <t>Component list</t>
   </si>
@@ -323,9 +322,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>Bill of Materials for Project [Ezlo-Radar-Sensor.PrjPcb]</t>
-  </si>
-  <si>
     <t>Ezlo-Radar-Sensor</t>
   </si>
   <si>
@@ -351,18 +347,45 @@
   </si>
   <si>
     <t>C7, C12, C14, C15</t>
+  </si>
+  <si>
+    <t>MICROPHONE</t>
+  </si>
+  <si>
+    <t>Mk1</t>
+  </si>
+  <si>
+    <t>Mic Omni-Directional -26dB 3.63V Rectangular Solder Pad T/R</t>
+  </si>
+  <si>
+    <t>ICS-43434</t>
+  </si>
+  <si>
+    <t>TDK InvenSense</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>Integrated Gesture Recognition Sensor with I2C Interface</t>
+  </si>
+  <si>
+    <t>PAJ7620U2</t>
+  </si>
+  <si>
+    <t>PixART Imaging Inc.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -522,8 +545,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -544,18 +574,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="1" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -813,12 +837,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -886,10 +923,10 @@
     <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -917,16 +954,7 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -949,18 +977,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="166" fontId="15" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -976,97 +1001,52 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="15" fillId="3" borderId="21" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1109,44 +1089,74 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1542,9 +1552,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S22"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -1578,15 +1588,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="91"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="72"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1596,8 +1606,8 @@
         <v>0</v>
       </c>
       <c r="E2" s="11"/>
-      <c r="F2" s="55" t="s">
-        <v>108</v>
+      <c r="F2" s="51" t="s">
+        <v>107</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -1621,8 +1631,8 @@
         <v>1</v>
       </c>
       <c r="E3" s="13"/>
-      <c r="F3" s="56" t="s">
-        <v>101</v>
+      <c r="F3" s="52" t="s">
+        <v>100</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -1636,7 +1646,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="92"/>
+      <c r="S3" s="73"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1646,8 +1656,8 @@
         <v>2</v>
       </c>
       <c r="E4" s="13"/>
-      <c r="F4" s="57" t="s">
-        <v>101</v>
+      <c r="F4" s="53" t="s">
+        <v>100</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -1661,7 +1671,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="93"/>
+      <c r="S4" s="74"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1671,7 +1681,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="13"/>
-      <c r="F5" s="58" t="s">
+      <c r="F5" s="54" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="15"/>
@@ -1686,7 +1696,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="93"/>
+      <c r="S5" s="74"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1707,7 +1717,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="93"/>
+      <c r="S6" s="74"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1728,7 +1738,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="93"/>
+      <c r="S7" s="74"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1749,7 +1759,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="93"/>
+      <c r="S8" s="74"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1780,10 +1790,10 @@
       <c r="J9" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="55" t="s">
         <v>91</v>
       </c>
-      <c r="L9" s="59" t="s">
+      <c r="L9" s="55" t="s">
         <v>89</v>
       </c>
       <c r="M9" s="30" t="s">
@@ -1810,183 +1820,183 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="50">
+      <c r="B10" s="47">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="108" t="s">
+      <c r="C10" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="109" t="s">
+      <c r="D10" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="109" t="s">
+      <c r="E10" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="110" t="s">
+      <c r="F10" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="G10" s="109" t="s">
+      <c r="G10" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="H10" s="110" t="s">
+      <c r="H10" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="I10" s="109" t="s">
+      <c r="I10" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="J10" s="110" t="s">
+      <c r="J10" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="K10" s="109" t="s">
+      <c r="K10" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="L10" s="110">
+      <c r="L10" s="39">
         <v>8</v>
       </c>
-      <c r="M10" s="109">
+      <c r="M10" s="38">
         <f>L10*10</f>
         <v>80</v>
       </c>
-      <c r="N10" s="110">
+      <c r="N10" s="39">
         <v>100</v>
       </c>
-      <c r="O10" s="111" t="s">
-        <v>103</v>
-      </c>
-      <c r="P10" s="112">
+      <c r="O10" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P10" s="49">
         <v>2E-3</v>
       </c>
-      <c r="Q10" s="113">
+      <c r="Q10" s="40">
         <f>P10*N10</f>
         <v>0.2</v>
       </c>
-      <c r="R10" s="109"/>
-      <c r="S10" s="114"/>
+      <c r="R10" s="38"/>
+      <c r="S10" s="83"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="51">
-        <f t="shared" ref="B11:B20" si="0">ROW(B11) - ROW($B$9)</f>
+      <c r="B11" s="48">
+        <f t="shared" ref="B11:B22" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="102" t="s">
+      <c r="C11" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="103" t="s">
+      <c r="D11" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="103" t="s">
+      <c r="E11" s="66" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="104" t="s">
+      <c r="F11" s="67" t="s">
         <v>42</v>
       </c>
-      <c r="G11" s="103" t="s">
+      <c r="G11" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="104" t="s">
+      <c r="H11" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="I11" s="103" t="s">
+      <c r="I11" s="66" t="s">
         <v>99</v>
       </c>
-      <c r="J11" s="104" t="s">
+      <c r="J11" s="67" t="s">
         <v>71</v>
       </c>
-      <c r="K11" s="103" t="s">
+      <c r="K11" s="66" t="s">
         <v>81</v>
       </c>
-      <c r="L11" s="104">
+      <c r="L11" s="67">
         <v>1</v>
       </c>
-      <c r="M11" s="103">
-        <f t="shared" ref="M11:M20" si="1">L11*10</f>
+      <c r="M11" s="66">
+        <f t="shared" ref="M11:M22" si="1">L11*10</f>
         <v>10</v>
       </c>
-      <c r="N11" s="104">
+      <c r="N11" s="67">
         <v>100</v>
       </c>
-      <c r="O11" s="105" t="s">
-        <v>103</v>
-      </c>
-      <c r="P11" s="106">
+      <c r="O11" s="68" t="s">
+        <v>102</v>
+      </c>
+      <c r="P11" s="69">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="Q11" s="107">
+      <c r="Q11" s="70">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
         <v>0.12</v>
       </c>
-      <c r="R11" s="103"/>
-      <c r="S11" s="103"/>
+      <c r="R11" s="66"/>
+      <c r="S11" s="66"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="50">
+      <c r="B12" s="47">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="108" t="s">
+      <c r="C12" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="109" t="s">
+      <c r="D12" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="109" t="s">
+      <c r="E12" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="110" t="s">
+      <c r="F12" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="109" t="s">
+      <c r="G12" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H12" s="110" t="s">
+      <c r="H12" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="I12" s="109" t="s">
+      <c r="I12" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="J12" s="110" t="s">
+      <c r="J12" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="K12" s="109" t="s">
+      <c r="K12" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="L12" s="110">
+      <c r="L12" s="39">
         <v>2</v>
       </c>
-      <c r="M12" s="109">
+      <c r="M12" s="38">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N12" s="110">
+      <c r="N12" s="39">
         <v>40</v>
       </c>
-      <c r="O12" s="111" t="s">
-        <v>103</v>
-      </c>
-      <c r="P12" s="112">
+      <c r="O12" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P12" s="49">
         <v>4.19E-2</v>
       </c>
-      <c r="Q12" s="113">
+      <c r="Q12" s="40">
         <f>P12*N12</f>
         <v>1.6759999999999999</v>
       </c>
-      <c r="R12" s="109"/>
-      <c r="S12" s="109"/>
+      <c r="R12" s="38"/>
+      <c r="S12" s="38"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="50">
+      <c r="B13" s="47">
         <f>ROW(B13) - ROW($B$9)</f>
         <v>4</v>
       </c>
-      <c r="C13" s="61" t="s">
+      <c r="C13" s="56" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E13" s="38" t="s">
         <v>33</v>
@@ -2019,13 +2029,13 @@
       <c r="N13" s="39">
         <v>50</v>
       </c>
-      <c r="O13" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P13" s="52">
+      <c r="O13" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P13" s="49">
         <v>9.9000000000000008E-3</v>
       </c>
-      <c r="Q13" s="42">
+      <c r="Q13" s="40">
         <f>P13*N13</f>
         <v>0.49500000000000005</v>
       </c>
@@ -2034,67 +2044,67 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="51">
+      <c r="B14" s="48">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="62" t="s">
+      <c r="C14" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="40" t="s">
+      <c r="E14" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="41" t="s">
+      <c r="F14" s="67" t="s">
         <v>42</v>
       </c>
-      <c r="G14" s="40" t="s">
+      <c r="G14" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="H14" s="41" t="s">
+      <c r="H14" s="67" t="s">
         <v>63</v>
       </c>
-      <c r="I14" s="40" t="s">
+      <c r="I14" s="66" t="s">
         <v>99</v>
       </c>
-      <c r="J14" s="41" t="s">
+      <c r="J14" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="K14" s="40" t="s">
+      <c r="K14" s="66" t="s">
         <v>84</v>
       </c>
-      <c r="L14" s="41">
+      <c r="L14" s="67">
         <v>1</v>
       </c>
-      <c r="M14" s="40">
+      <c r="M14" s="66">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N14" s="41">
+      <c r="N14" s="67">
         <v>20</v>
       </c>
-      <c r="O14" s="66" t="s">
-        <v>103</v>
-      </c>
-      <c r="P14" s="53">
+      <c r="O14" s="68" t="s">
+        <v>102</v>
+      </c>
+      <c r="P14" s="69">
         <v>2.5600000000000001E-2</v>
       </c>
-      <c r="Q14" s="43">
+      <c r="Q14" s="70">
         <f t="shared" ref="Q14" si="3">P14*N14</f>
         <v>0.51200000000000001</v>
       </c>
-      <c r="R14" s="40"/>
-      <c r="S14" s="40"/>
+      <c r="R14" s="66"/>
+      <c r="S14" s="66"/>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="50">
+      <c r="B15" s="47">
         <f>ROW(B15) - ROW($B$9)</f>
         <v>6</v>
       </c>
-      <c r="C15" s="61" t="s">
+      <c r="C15" s="56" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="38" t="s">
@@ -2131,13 +2141,13 @@
       <c r="N15" s="39">
         <v>100</v>
       </c>
-      <c r="O15" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P15" s="52">
+      <c r="O15" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P15" s="49">
         <v>6.6E-3</v>
       </c>
-      <c r="Q15" s="42">
+      <c r="Q15" s="40">
         <f>P15*N15</f>
         <v>0.66</v>
       </c>
@@ -2146,67 +2156,67 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="51">
+      <c r="B16" s="48">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="C16" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="40" t="s">
+      <c r="E16" s="66" t="s">
         <v>36</v>
       </c>
-      <c r="F16" s="41" t="s">
+      <c r="F16" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="40" t="s">
+      <c r="G16" s="66" t="s">
         <v>56</v>
       </c>
-      <c r="H16" s="41" t="s">
+      <c r="H16" s="67" t="s">
         <v>64</v>
       </c>
-      <c r="I16" s="40" t="s">
+      <c r="I16" s="66" t="s">
         <v>99</v>
       </c>
-      <c r="J16" s="41" t="s">
+      <c r="J16" s="67" t="s">
         <v>77</v>
       </c>
-      <c r="K16" s="40" t="s">
+      <c r="K16" s="66" t="s">
         <v>86</v>
       </c>
-      <c r="L16" s="41">
+      <c r="L16" s="67">
         <v>7</v>
       </c>
-      <c r="M16" s="40">
+      <c r="M16" s="66">
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="N16" s="41">
+      <c r="N16" s="67">
         <v>100</v>
       </c>
-      <c r="O16" s="66" t="s">
-        <v>103</v>
-      </c>
-      <c r="P16" s="53">
+      <c r="O16" s="68" t="s">
+        <v>102</v>
+      </c>
+      <c r="P16" s="69">
         <v>5.7000000000000002E-3</v>
       </c>
-      <c r="Q16" s="43">
+      <c r="Q16" s="70">
         <f t="shared" ref="Q16" si="4">P16*N16</f>
         <v>0.57000000000000006</v>
       </c>
-      <c r="R16" s="40"/>
-      <c r="S16" s="40"/>
+      <c r="R16" s="66"/>
+      <c r="S16" s="66"/>
     </row>
     <row r="17" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="50">
+      <c r="B17" s="47">
         <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
-      <c r="C17" s="64" t="s">
+      <c r="C17" s="57" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="38" t="s">
@@ -2216,7 +2226,7 @@
         <v>37</v>
       </c>
       <c r="F17" s="39" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G17" s="38" t="s">
         <v>45</v>
@@ -2243,241 +2253,337 @@
       <c r="N17" s="39">
         <v>61</v>
       </c>
-      <c r="O17" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P17" s="52">
+      <c r="O17" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P17" s="49">
         <v>9.1499999999999998E-2</v>
       </c>
-      <c r="Q17" s="42">
+      <c r="Q17" s="40">
         <f>P17*N17</f>
         <v>5.5815000000000001</v>
       </c>
       <c r="R17" s="38"/>
       <c r="S17" s="38"/>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="51">
-        <f t="shared" si="0"/>
+      <c r="B18" s="47">
+        <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="63" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="40" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="F18" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="G18" s="40" t="s">
-        <v>57</v>
-      </c>
-      <c r="H18" s="41" t="s">
-        <v>66</v>
-      </c>
-      <c r="I18" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="J18" s="41" t="s">
-        <v>79</v>
-      </c>
-      <c r="K18" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="L18" s="41">
+      <c r="C18" s="90" t="s">
+        <v>109</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>110</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="F18" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="G18" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="I18" s="38"/>
+      <c r="J18" s="38"/>
+      <c r="K18" s="38"/>
+      <c r="L18" s="38">
         <v>1</v>
       </c>
-      <c r="M18" s="40">
+      <c r="M18" s="38">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N18" s="41">
-        <v>50</v>
-      </c>
-      <c r="O18" s="66" t="s">
-        <v>103</v>
-      </c>
-      <c r="P18" s="53">
-        <v>4.1999999999999997E-3</v>
-      </c>
-      <c r="Q18" s="43">
-        <f t="shared" ref="Q18" si="5">P18*N18</f>
-        <v>0.21</v>
-      </c>
-      <c r="R18" s="40"/>
-      <c r="S18" s="40"/>
+      <c r="N18" s="38">
+        <v>11</v>
+      </c>
+      <c r="O18" s="38"/>
+      <c r="P18" s="40"/>
+      <c r="Q18" s="40">
+        <f>P18*N18</f>
+        <v>0</v>
+      </c>
+      <c r="R18" s="38"/>
+      <c r="S18" s="91"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="50">
-        <f>ROW(B19) - ROW($B$9)</f>
+      <c r="B19" s="48">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="64" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>47</v>
-      </c>
-      <c r="G19" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="H19" s="39" t="s">
-        <v>67</v>
-      </c>
-      <c r="I19" s="38" t="s">
+      <c r="C19" s="84" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="66" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="66" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" s="67" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" s="66" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="67" t="s">
+        <v>66</v>
+      </c>
+      <c r="I19" s="66" t="s">
         <v>99</v>
       </c>
-      <c r="J19" s="39"/>
-      <c r="K19" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="L19" s="39">
+      <c r="J19" s="67" t="s">
+        <v>79</v>
+      </c>
+      <c r="K19" s="66" t="s">
+        <v>87</v>
+      </c>
+      <c r="L19" s="67">
         <v>1</v>
       </c>
-      <c r="M19" s="38">
+      <c r="M19" s="66">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N19" s="39"/>
-      <c r="O19" s="38"/>
-      <c r="P19" s="52"/>
-      <c r="Q19" s="42">
-        <f>P19*N19</f>
-        <v>0</v>
-      </c>
-      <c r="R19" s="38"/>
-      <c r="S19" s="38"/>
-    </row>
-    <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N19" s="67">
+        <v>50</v>
+      </c>
+      <c r="O19" s="68" t="s">
+        <v>102</v>
+      </c>
+      <c r="P19" s="69">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="Q19" s="70">
+        <f t="shared" ref="Q19" si="5">P19*N19</f>
+        <v>0.21</v>
+      </c>
+      <c r="R19" s="66"/>
+      <c r="S19" s="66"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="85">
-        <f t="shared" si="0"/>
+      <c r="B20" s="47">
+        <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="86" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" s="60" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="60" t="s">
-        <v>40</v>
-      </c>
-      <c r="F20" s="87" t="s">
-        <v>102</v>
-      </c>
-      <c r="G20" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="H20" s="87" t="s">
-        <v>68</v>
-      </c>
-      <c r="I20" s="60" t="s">
+      <c r="C20" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="I20" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="J20" s="87"/>
-      <c r="K20" s="60" t="s">
-        <v>88</v>
-      </c>
-      <c r="L20" s="87">
+      <c r="J20" s="39"/>
+      <c r="K20" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="L20" s="39">
         <v>1</v>
       </c>
-      <c r="M20" s="60">
+      <c r="M20" s="38">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N20" s="87"/>
-      <c r="O20" s="60"/>
-      <c r="P20" s="88"/>
-      <c r="Q20" s="89">
-        <f t="shared" ref="Q20" si="6">P20*N20</f>
+      <c r="N20" s="39">
+        <v>11</v>
+      </c>
+      <c r="O20" s="38"/>
+      <c r="P20" s="49"/>
+      <c r="Q20" s="40">
+        <f>P20*N20</f>
         <v>0</v>
       </c>
-      <c r="R20" s="60"/>
-      <c r="S20" s="60"/>
-    </row>
-    <row r="21" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R20" s="38"/>
+      <c r="S20" s="38"/>
+    </row>
+    <row r="21" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="44"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="49"/>
-      <c r="J21" s="48"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="49"/>
-      <c r="N21" s="98" t="s">
+      <c r="B21" s="48">
+        <f t="shared" ref="B21" si="6">ROW(B21) - ROW($B$9)</f>
+        <v>12</v>
+      </c>
+      <c r="C21" s="92" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="66" t="s">
+        <v>114</v>
+      </c>
+      <c r="E21" s="66" t="s">
+        <v>115</v>
+      </c>
+      <c r="F21" s="66" t="s">
+        <v>101</v>
+      </c>
+      <c r="G21" s="66" t="s">
+        <v>116</v>
+      </c>
+      <c r="H21" s="66" t="s">
+        <v>117</v>
+      </c>
+      <c r="I21" s="66"/>
+      <c r="J21" s="66"/>
+      <c r="K21" s="66"/>
+      <c r="L21" s="66">
+        <v>1</v>
+      </c>
+      <c r="M21" s="38">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N21" s="66">
+        <v>11</v>
+      </c>
+      <c r="O21" s="66"/>
+      <c r="P21" s="70"/>
+      <c r="Q21" s="70">
+        <f t="shared" ref="Q21" si="7">P21*N21</f>
+        <v>0</v>
+      </c>
+      <c r="R21" s="66"/>
+      <c r="S21" s="91"/>
+    </row>
+    <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1"/>
+      <c r="B22" s="64">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="C22" s="85" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="86" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="86" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" s="87" t="s">
+        <v>101</v>
+      </c>
+      <c r="G22" s="86" t="s">
+        <v>59</v>
+      </c>
+      <c r="H22" s="87" t="s">
+        <v>68</v>
+      </c>
+      <c r="I22" s="86" t="s">
+        <v>99</v>
+      </c>
+      <c r="J22" s="87"/>
+      <c r="K22" s="86" t="s">
+        <v>88</v>
+      </c>
+      <c r="L22" s="87">
+        <v>1</v>
+      </c>
+      <c r="M22" s="86">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N22" s="87">
+        <v>11</v>
+      </c>
+      <c r="O22" s="86"/>
+      <c r="P22" s="88"/>
+      <c r="Q22" s="89">
+        <f t="shared" ref="Q22" si="8">P22*N22</f>
+        <v>0</v>
+      </c>
+      <c r="R22" s="86"/>
+      <c r="S22" s="86"/>
+    </row>
+    <row r="23" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="45"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="45"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="46"/>
+      <c r="N23" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="O21" s="99"/>
-      <c r="P21" s="99"/>
-      <c r="Q21" s="79">
-        <f>SUM(Q10:Q20)</f>
+      <c r="O23" s="80"/>
+      <c r="P23" s="80"/>
+      <c r="Q23" s="62">
+        <f>SUM(Q10:Q22)</f>
         <v>10.024500000000002</v>
       </c>
-      <c r="R21" s="94"/>
-      <c r="S21" s="95"/>
-    </row>
-    <row r="22" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="100" t="s">
+      <c r="R23" s="75"/>
+      <c r="S23" s="76"/>
+    </row>
+    <row r="24" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="81" t="s">
         <v>6</v>
       </c>
-      <c r="O22" s="101"/>
-      <c r="P22" s="101"/>
-      <c r="Q22" s="54">
-        <f>Q21/10</f>
+      <c r="O24" s="82"/>
+      <c r="P24" s="82"/>
+      <c r="Q24" s="50">
+        <f>Q23/10</f>
         <v>1.0024500000000001</v>
       </c>
-      <c r="R22" s="96"/>
-      <c r="S22" s="97"/>
+      <c r="R24" s="77"/>
+      <c r="S24" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="R21:S22"/>
-    <mergeCell ref="N21:P21"/>
-    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="R23:S24"/>
+    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="N24:P24"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O10" r:id="rId1" xr:uid="{8D2FB7B3-5497-4892-94A0-685942AD8F20}"/>
-    <hyperlink ref="O11" r:id="rId2" xr:uid="{897FE6A0-A0CD-4ECE-84EA-106137AD5E12}"/>
-    <hyperlink ref="O12" r:id="rId3" xr:uid="{ABE5FD74-F03F-4668-BCEA-2CCADC820A1C}"/>
-    <hyperlink ref="O13" r:id="rId4" xr:uid="{C0441405-5450-4B44-A768-136FBA22E13D}"/>
-    <hyperlink ref="O14" r:id="rId5" xr:uid="{997A6499-8A85-4F11-A1C0-659F37BCDF47}"/>
-    <hyperlink ref="O15" r:id="rId6" xr:uid="{B2B4B4D1-3621-40F1-BAA1-56709C1EB6B3}"/>
-    <hyperlink ref="O16" r:id="rId7" xr:uid="{3B72AF33-B920-4BFB-ADC6-8D72FDD02BDA}"/>
-    <hyperlink ref="O17" r:id="rId8" xr:uid="{123B586C-4B24-4DA7-9E7B-AEB3318E9AC5}"/>
-    <hyperlink ref="O18" r:id="rId9" xr:uid="{51846484-CE84-40DA-AF1B-26D70B22E9C3}"/>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O12" r:id="rId3"/>
+    <hyperlink ref="O13" r:id="rId4"/>
+    <hyperlink ref="O14" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O16" r:id="rId7"/>
+    <hyperlink ref="O17" r:id="rId8"/>
+    <hyperlink ref="O19" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
@@ -2486,8 +2592,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC3D942-A413-440E-98EA-CC95081980EF}">
-  <dimension ref="A1:S23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -2521,15 +2627,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="91"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="72"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2539,8 +2645,8 @@
         <v>0</v>
       </c>
       <c r="E2" s="11"/>
-      <c r="F2" s="55" t="s">
-        <v>100</v>
+      <c r="F2" s="51" t="s">
+        <v>107</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -2564,8 +2670,8 @@
         <v>1</v>
       </c>
       <c r="E3" s="13"/>
-      <c r="F3" s="56" t="s">
-        <v>101</v>
+      <c r="F3" s="52" t="s">
+        <v>100</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -2579,7 +2685,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="92"/>
+      <c r="S3" s="73"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2589,8 +2695,8 @@
         <v>2</v>
       </c>
       <c r="E4" s="13"/>
-      <c r="F4" s="57" t="s">
-        <v>101</v>
+      <c r="F4" s="53" t="s">
+        <v>100</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -2604,7 +2710,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="93"/>
+      <c r="S4" s="74"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2614,7 +2720,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="13"/>
-      <c r="F5" s="58" t="s">
+      <c r="F5" s="54" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="15"/>
@@ -2629,7 +2735,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="93"/>
+      <c r="S5" s="74"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2650,7 +2756,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="93"/>
+      <c r="S6" s="74"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2671,7 +2777,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="93"/>
+      <c r="S7" s="74"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2692,7 +2798,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="93"/>
+      <c r="S8" s="74"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2723,26 +2829,26 @@
       <c r="J9" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="55" t="s">
         <v>91</v>
       </c>
-      <c r="L9" s="59" t="s">
+      <c r="L9" s="55" t="s">
         <v>89</v>
       </c>
       <c r="M9" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="N9" s="31" t="s">
         <v>104</v>
-      </c>
-      <c r="N9" s="31" t="s">
-        <v>105</v>
       </c>
       <c r="O9" s="30" t="s">
         <v>94</v>
       </c>
       <c r="P9" s="31" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="R9" s="31" t="s">
         <v>97</v>
@@ -2751,13 +2857,13 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:19" s="69" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="67"/>
-      <c r="B10" s="50">
+    <row r="10" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="59"/>
+      <c r="B10" s="47">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="61" t="s">
+      <c r="C10" s="56" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="38" t="s">
@@ -2794,82 +2900,82 @@
       <c r="N10" s="39">
         <v>8100</v>
       </c>
-      <c r="O10" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P10" s="52">
+      <c r="O10" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P10" s="49">
         <v>1.4E-3</v>
       </c>
-      <c r="Q10" s="42">
+      <c r="Q10" s="40">
         <f>P10*N10</f>
         <v>11.34</v>
       </c>
       <c r="R10" s="39"/>
-      <c r="S10" s="68"/>
+      <c r="S10" s="93"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="70">
-        <f t="shared" ref="B11:B21" si="0">ROW(B11) - ROW($B$9)</f>
+      <c r="B11" s="61">
+        <f t="shared" ref="B11:B23" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="77" t="s">
+      <c r="C11" s="94" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="72" t="s">
+      <c r="D11" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="95" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="73" t="s">
+      <c r="F11" s="96" t="s">
         <v>42</v>
       </c>
-      <c r="G11" s="72" t="s">
+      <c r="G11" s="95" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="73" t="s">
+      <c r="H11" s="96" t="s">
         <v>61</v>
       </c>
-      <c r="I11" s="72" t="s">
+      <c r="I11" s="95" t="s">
         <v>99</v>
       </c>
-      <c r="J11" s="73" t="s">
+      <c r="J11" s="96" t="s">
         <v>71</v>
       </c>
-      <c r="K11" s="72" t="s">
+      <c r="K11" s="95" t="s">
         <v>81</v>
       </c>
-      <c r="L11" s="73">
+      <c r="L11" s="96">
         <v>1</v>
       </c>
-      <c r="M11" s="72">
-        <f t="shared" ref="M11:M21" si="1">L11*1000</f>
+      <c r="M11" s="95">
+        <f t="shared" ref="M11:M23" si="1">L11*1000</f>
         <v>1000</v>
       </c>
-      <c r="N11" s="73">
+      <c r="N11" s="96">
         <v>1100</v>
       </c>
-      <c r="O11" s="74" t="s">
-        <v>103</v>
-      </c>
-      <c r="P11" s="75">
+      <c r="O11" s="97" t="s">
+        <v>102</v>
+      </c>
+      <c r="P11" s="98">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="Q11" s="76">
+      <c r="Q11" s="99">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
         <v>0.99</v>
       </c>
-      <c r="R11" s="73"/>
-      <c r="S11" s="72"/>
-    </row>
-    <row r="12" spans="1:19" s="69" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="67"/>
-      <c r="B12" s="50">
+      <c r="R11" s="96"/>
+      <c r="S11" s="95"/>
+    </row>
+    <row r="12" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="59"/>
+      <c r="B12" s="47">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="61" t="s">
+      <c r="C12" s="56" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="38" t="s">
@@ -2906,82 +3012,82 @@
       <c r="N12" s="39">
         <v>2060</v>
       </c>
-      <c r="O12" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P12" s="52">
+      <c r="O12" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P12" s="49">
         <v>3.1199999999999999E-2</v>
       </c>
-      <c r="Q12" s="42">
+      <c r="Q12" s="40">
         <f>P12*N12</f>
         <v>64.271999999999991</v>
       </c>
       <c r="R12" s="39"/>
       <c r="S12" s="38"/>
     </row>
-    <row r="13" spans="1:19" s="69" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="67"/>
-      <c r="B13" s="51">
+    <row r="13" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="59"/>
+      <c r="B13" s="48">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="62" t="s">
+      <c r="C13" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="40" t="s">
+      <c r="E13" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="41" t="s">
+      <c r="F13" s="67" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="40" t="s">
+      <c r="G13" s="66" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="41" t="s">
+      <c r="H13" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="I13" s="40" t="s">
+      <c r="I13" s="66" t="s">
         <v>99</v>
       </c>
-      <c r="J13" s="41" t="s">
+      <c r="J13" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="K13" s="40" t="s">
+      <c r="K13" s="66" t="s">
         <v>83</v>
       </c>
-      <c r="L13" s="41">
+      <c r="L13" s="67">
         <v>1</v>
       </c>
-      <c r="M13" s="40">
+      <c r="M13" s="66">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N13" s="41">
+      <c r="N13" s="67">
         <v>1060</v>
       </c>
-      <c r="O13" s="66" t="s">
-        <v>103</v>
-      </c>
-      <c r="P13" s="53">
+      <c r="O13" s="68" t="s">
+        <v>102</v>
+      </c>
+      <c r="P13" s="69">
         <v>1.7299999999999999E-2</v>
       </c>
-      <c r="Q13" s="43">
+      <c r="Q13" s="70">
         <f t="shared" ref="Q13" si="3">P13*N13</f>
         <v>18.338000000000001</v>
       </c>
-      <c r="R13" s="41"/>
-      <c r="S13" s="40"/>
-    </row>
-    <row r="14" spans="1:19" s="69" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="67"/>
-      <c r="B14" s="50">
+      <c r="R13" s="67"/>
+      <c r="S13" s="66"/>
+    </row>
+    <row r="14" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="59"/>
+      <c r="B14" s="47">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="61" t="s">
+      <c r="C14" s="56" t="s">
         <v>9</v>
       </c>
       <c r="D14" s="38" t="s">
@@ -3018,13 +3124,13 @@
       <c r="N14" s="39">
         <v>3050</v>
       </c>
-      <c r="O14" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P14" s="52">
+      <c r="O14" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P14" s="49">
         <v>6.7999999999999996E-3</v>
       </c>
-      <c r="Q14" s="42">
+      <c r="Q14" s="40">
         <f>P14*N14</f>
         <v>20.74</v>
       </c>
@@ -3033,67 +3139,67 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="70">
+      <c r="B15" s="61">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="77" t="s">
+      <c r="C15" s="94" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="72" t="s">
+      <c r="D15" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="72" t="s">
+      <c r="E15" s="95" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="73" t="s">
+      <c r="F15" s="96" t="s">
         <v>42</v>
       </c>
-      <c r="G15" s="72" t="s">
+      <c r="G15" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="H15" s="73" t="s">
+      <c r="H15" s="96" t="s">
         <v>63</v>
       </c>
-      <c r="I15" s="72" t="s">
+      <c r="I15" s="95" t="s">
         <v>99</v>
       </c>
-      <c r="J15" s="73" t="s">
+      <c r="J15" s="96" t="s">
         <v>75</v>
       </c>
-      <c r="K15" s="72" t="s">
+      <c r="K15" s="95" t="s">
         <v>84</v>
       </c>
-      <c r="L15" s="73">
+      <c r="L15" s="96">
         <v>1</v>
       </c>
-      <c r="M15" s="72">
+      <c r="M15" s="95">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N15" s="73">
+      <c r="N15" s="96">
         <v>1080</v>
       </c>
-      <c r="O15" s="74" t="s">
-        <v>103</v>
-      </c>
-      <c r="P15" s="75">
+      <c r="O15" s="97" t="s">
+        <v>102</v>
+      </c>
+      <c r="P15" s="98">
         <v>1.7829999999999999E-2</v>
       </c>
-      <c r="Q15" s="76">
+      <c r="Q15" s="99">
         <f t="shared" ref="Q15" si="4">P15*N15</f>
         <v>19.256399999999999</v>
       </c>
-      <c r="R15" s="73"/>
-      <c r="S15" s="72"/>
-    </row>
-    <row r="16" spans="1:19" s="69" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="67"/>
-      <c r="B16" s="50">
+      <c r="R15" s="96"/>
+      <c r="S15" s="95"/>
+    </row>
+    <row r="16" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="59"/>
+      <c r="B16" s="47">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="61" t="s">
+      <c r="C16" s="56" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="38" t="s">
@@ -3130,13 +3236,13 @@
       <c r="N16" s="39">
         <v>1100</v>
       </c>
-      <c r="O16" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P16" s="52">
+      <c r="O16" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P16" s="49">
         <v>5.5999999999999999E-3</v>
       </c>
-      <c r="Q16" s="42">
+      <c r="Q16" s="40">
         <f>P16*N16</f>
         <v>6.16</v>
       </c>
@@ -3145,67 +3251,67 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="70">
+      <c r="B17" s="61">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="71" t="s">
+      <c r="C17" s="100" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="72" t="s">
+      <c r="D17" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="72" t="s">
+      <c r="E17" s="95" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="73" t="s">
+      <c r="F17" s="96" t="s">
         <v>44</v>
       </c>
-      <c r="G17" s="72" t="s">
+      <c r="G17" s="95" t="s">
         <v>56</v>
       </c>
-      <c r="H17" s="73" t="s">
+      <c r="H17" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="I17" s="72" t="s">
+      <c r="I17" s="95" t="s">
         <v>99</v>
       </c>
-      <c r="J17" s="73" t="s">
+      <c r="J17" s="96" t="s">
         <v>77</v>
       </c>
-      <c r="K17" s="72" t="s">
+      <c r="K17" s="95" t="s">
         <v>86</v>
       </c>
-      <c r="L17" s="73">
+      <c r="L17" s="96">
         <v>7</v>
       </c>
-      <c r="M17" s="72">
+      <c r="M17" s="95">
         <f t="shared" si="1"/>
         <v>7000</v>
       </c>
-      <c r="N17" s="73">
+      <c r="N17" s="96">
         <v>7100</v>
       </c>
-      <c r="O17" s="74" t="s">
-        <v>103</v>
-      </c>
-      <c r="P17" s="75">
+      <c r="O17" s="97" t="s">
+        <v>102</v>
+      </c>
+      <c r="P17" s="98">
         <v>4.1000000000000003E-3</v>
       </c>
-      <c r="Q17" s="76">
+      <c r="Q17" s="99">
         <f t="shared" ref="Q17" si="5">P17*N17</f>
         <v>29.110000000000003</v>
       </c>
-      <c r="R17" s="73"/>
-      <c r="S17" s="72"/>
-    </row>
-    <row r="18" spans="1:19" s="69" customFormat="1" ht="48" x14ac:dyDescent="0.25">
-      <c r="A18" s="67"/>
-      <c r="B18" s="50">
+      <c r="R17" s="96"/>
+      <c r="S17" s="95"/>
+    </row>
+    <row r="18" spans="1:19" s="60" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A18" s="59"/>
+      <c r="B18" s="47">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="64" t="s">
+      <c r="C18" s="57" t="s">
         <v>11</v>
       </c>
       <c r="D18" s="38" t="s">
@@ -3215,7 +3321,7 @@
         <v>37</v>
       </c>
       <c r="F18" s="39" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G18" s="38" t="s">
         <v>45</v>
@@ -3242,242 +3348,330 @@
       <c r="N18" s="39">
         <v>1098</v>
       </c>
-      <c r="O18" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="P18" s="52">
+      <c r="O18" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="P18" s="49">
         <v>7.4399999999999994E-2</v>
       </c>
-      <c r="Q18" s="42">
+      <c r="Q18" s="40">
         <f>P18*N18</f>
         <v>81.691199999999995</v>
       </c>
       <c r="R18" s="39"/>
       <c r="S18" s="38"/>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="70">
-        <f t="shared" si="0"/>
+      <c r="B19" s="47">
+        <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="71" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="72" t="s">
-        <v>25</v>
-      </c>
-      <c r="E19" s="72" t="s">
-        <v>38</v>
-      </c>
-      <c r="F19" s="73" t="s">
-        <v>46</v>
-      </c>
-      <c r="G19" s="72" t="s">
-        <v>57</v>
-      </c>
-      <c r="H19" s="73" t="s">
-        <v>66</v>
-      </c>
-      <c r="I19" s="72" t="s">
-        <v>99</v>
-      </c>
-      <c r="J19" s="73" t="s">
-        <v>79</v>
-      </c>
-      <c r="K19" s="72" t="s">
-        <v>87</v>
-      </c>
-      <c r="L19" s="73">
+      <c r="C19" s="90" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="G19" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="H19" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="I19" s="38"/>
+      <c r="J19" s="38"/>
+      <c r="K19" s="38"/>
+      <c r="L19" s="38">
         <v>1</v>
       </c>
-      <c r="M19" s="72">
+      <c r="M19" s="38">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N19" s="73">
-        <v>1050</v>
-      </c>
-      <c r="O19" s="74" t="s">
-        <v>103</v>
-      </c>
-      <c r="P19" s="75">
-        <v>3.5000000000000001E-3</v>
-      </c>
-      <c r="Q19" s="76">
-        <f t="shared" ref="Q19" si="6">P19*N19</f>
-        <v>3.6750000000000003</v>
-      </c>
-      <c r="R19" s="73"/>
-      <c r="S19" s="72"/>
-    </row>
-    <row r="20" spans="1:19" s="69" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="67"/>
-      <c r="B20" s="50">
-        <f>ROW(B20) - ROW($B$9)</f>
+      <c r="N19" s="38"/>
+      <c r="O19" s="38"/>
+      <c r="P19" s="40"/>
+      <c r="Q19" s="40">
+        <f>P19*N19</f>
+        <v>0</v>
+      </c>
+      <c r="R19" s="38"/>
+      <c r="S19" s="91"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="61">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="64" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="F20" s="39" t="s">
-        <v>47</v>
-      </c>
-      <c r="G20" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="H20" s="39" t="s">
-        <v>67</v>
-      </c>
-      <c r="I20" s="38" t="s">
+      <c r="C20" s="100" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="95" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="95" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20" s="96" t="s">
+        <v>46</v>
+      </c>
+      <c r="G20" s="95" t="s">
+        <v>57</v>
+      </c>
+      <c r="H20" s="96" t="s">
+        <v>66</v>
+      </c>
+      <c r="I20" s="95" t="s">
         <v>99</v>
       </c>
-      <c r="J20" s="39"/>
-      <c r="K20" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="L20" s="39">
+      <c r="J20" s="96" t="s">
+        <v>79</v>
+      </c>
+      <c r="K20" s="95" t="s">
+        <v>87</v>
+      </c>
+      <c r="L20" s="96">
         <v>1</v>
       </c>
-      <c r="M20" s="38">
+      <c r="M20" s="95">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N20" s="39"/>
-      <c r="O20" s="38"/>
-      <c r="P20" s="52"/>
-      <c r="Q20" s="42">
-        <f>P20*N20</f>
-        <v>0</v>
-      </c>
-      <c r="R20" s="39"/>
-      <c r="S20" s="38"/>
-    </row>
-    <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-      <c r="B21" s="80">
-        <f t="shared" si="0"/>
+      <c r="N20" s="96">
+        <v>1050</v>
+      </c>
+      <c r="O20" s="97" t="s">
+        <v>102</v>
+      </c>
+      <c r="P20" s="98">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="Q20" s="99">
+        <f t="shared" ref="Q20" si="6">P20*N20</f>
+        <v>3.6750000000000003</v>
+      </c>
+      <c r="R20" s="96"/>
+      <c r="S20" s="95"/>
+    </row>
+    <row r="21" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="59"/>
+      <c r="B21" s="47">
+        <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="81" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="78" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21" s="78" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21" s="82" t="s">
-        <v>102</v>
-      </c>
-      <c r="G21" s="78" t="s">
-        <v>59</v>
-      </c>
-      <c r="H21" s="82" t="s">
-        <v>68</v>
-      </c>
-      <c r="I21" s="78" t="s">
+      <c r="C21" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="F21" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="H21" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="I21" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="J21" s="82"/>
-      <c r="K21" s="78" t="s">
-        <v>88</v>
-      </c>
-      <c r="L21" s="82">
+      <c r="J21" s="39"/>
+      <c r="K21" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="L21" s="39">
         <v>1</v>
       </c>
-      <c r="M21" s="78">
+      <c r="M21" s="38">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N21" s="82"/>
-      <c r="O21" s="78"/>
-      <c r="P21" s="83"/>
-      <c r="Q21" s="84">
-        <f t="shared" ref="Q21" si="7">P21*N21</f>
+      <c r="N21" s="39"/>
+      <c r="O21" s="38"/>
+      <c r="P21" s="49"/>
+      <c r="Q21" s="40">
+        <f>P21*N21</f>
         <v>0</v>
       </c>
-      <c r="R21" s="82"/>
-      <c r="S21" s="78"/>
-    </row>
-    <row r="22" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="39"/>
+      <c r="S21" s="38"/>
+    </row>
+    <row r="22" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="44"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="49"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="49"/>
-      <c r="J22" s="48"/>
-      <c r="K22" s="49"/>
-      <c r="L22" s="49"/>
-      <c r="M22" s="49"/>
-      <c r="N22" s="98" t="s">
+      <c r="B22" s="48">
+        <f t="shared" ref="B22" si="7">ROW(B22) - ROW($B$9)</f>
+        <v>13</v>
+      </c>
+      <c r="C22" s="92" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="66" t="s">
+        <v>114</v>
+      </c>
+      <c r="E22" s="66" t="s">
+        <v>115</v>
+      </c>
+      <c r="F22" s="66" t="s">
+        <v>101</v>
+      </c>
+      <c r="G22" s="66" t="s">
+        <v>116</v>
+      </c>
+      <c r="H22" s="66" t="s">
+        <v>117</v>
+      </c>
+      <c r="I22" s="66"/>
+      <c r="J22" s="66"/>
+      <c r="K22" s="66"/>
+      <c r="L22" s="66">
+        <v>1</v>
+      </c>
+      <c r="M22" s="38">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N22" s="66"/>
+      <c r="O22" s="66"/>
+      <c r="P22" s="70"/>
+      <c r="Q22" s="70">
+        <f t="shared" ref="Q22" si="8">P22*N22</f>
+        <v>0</v>
+      </c>
+      <c r="R22" s="66"/>
+      <c r="S22" s="91"/>
+    </row>
+    <row r="23" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1"/>
+      <c r="B23" s="63">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C23" s="101" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="102" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="103" t="s">
+        <v>101</v>
+      </c>
+      <c r="G23" s="102" t="s">
+        <v>59</v>
+      </c>
+      <c r="H23" s="103" t="s">
+        <v>68</v>
+      </c>
+      <c r="I23" s="102" t="s">
+        <v>99</v>
+      </c>
+      <c r="J23" s="103"/>
+      <c r="K23" s="102" t="s">
+        <v>88</v>
+      </c>
+      <c r="L23" s="103">
+        <v>1</v>
+      </c>
+      <c r="M23" s="102">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N23" s="103"/>
+      <c r="O23" s="102"/>
+      <c r="P23" s="104"/>
+      <c r="Q23" s="105">
+        <f t="shared" ref="Q23" si="9">P23*N23</f>
+        <v>0</v>
+      </c>
+      <c r="R23" s="103"/>
+      <c r="S23" s="102"/>
+    </row>
+    <row r="24" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="41"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="46"/>
+      <c r="J24" s="45"/>
+      <c r="K24" s="46"/>
+      <c r="L24" s="46"/>
+      <c r="M24" s="46"/>
+      <c r="N24" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="O22" s="99"/>
-      <c r="P22" s="99"/>
-      <c r="Q22" s="79">
-        <f>SUM(Q10:Q21)</f>
+      <c r="O24" s="80"/>
+      <c r="P24" s="80"/>
+      <c r="Q24" s="62">
+        <f>SUM(Q10:Q23)</f>
         <v>255.57260000000002</v>
       </c>
-      <c r="R22" s="94"/>
-      <c r="S22" s="95"/>
-    </row>
-    <row r="23" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="100" t="s">
+      <c r="R24" s="75"/>
+      <c r="S24" s="76"/>
+    </row>
+    <row r="25" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="1"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="81" t="s">
         <v>6</v>
       </c>
-      <c r="O23" s="101"/>
-      <c r="P23" s="101"/>
-      <c r="Q23" s="54">
-        <f>Q22/10</f>
+      <c r="O25" s="82"/>
+      <c r="P25" s="82"/>
+      <c r="Q25" s="50">
+        <f>Q24/10</f>
         <v>25.557260000000003</v>
       </c>
-      <c r="R23" s="96"/>
-      <c r="S23" s="97"/>
+      <c r="R25" s="77"/>
+      <c r="S25" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="R22:S23"/>
-    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="R24:S25"/>
+    <mergeCell ref="N25:P25"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O10" r:id="rId1" xr:uid="{824749A7-A10A-499A-8CD0-DF156B8FA5FC}"/>
-    <hyperlink ref="O11" r:id="rId2" xr:uid="{990546FC-1FDB-4492-B864-1BDF72FA22BE}"/>
-    <hyperlink ref="O12" r:id="rId3" xr:uid="{3000D653-7CAB-462E-8C3E-745C63F83C29}"/>
-    <hyperlink ref="O13" r:id="rId4" xr:uid="{B5E800E5-0082-4305-B79A-5444E5776F33}"/>
-    <hyperlink ref="O14" r:id="rId5" xr:uid="{346FAD4E-9664-4F35-B95F-63182E8A9027}"/>
-    <hyperlink ref="O15" r:id="rId6" xr:uid="{613783D1-65CD-4819-B8D8-C912FDC45FD2}"/>
-    <hyperlink ref="O16" r:id="rId7" xr:uid="{E93EE780-47B1-46B9-AC98-284620CAA4F5}"/>
-    <hyperlink ref="O17" r:id="rId8" xr:uid="{B03B7119-0357-469D-986A-CF49ADA570AD}"/>
-    <hyperlink ref="O18" r:id="rId9" xr:uid="{6D800400-3AC9-4EBE-9D21-937BB2ED76F3}"/>
-    <hyperlink ref="O19" r:id="rId10" xr:uid="{B44B5583-7655-4535-92B0-56130AAE3A53}"/>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O12" r:id="rId3"/>
+    <hyperlink ref="O13" r:id="rId4"/>
+    <hyperlink ref="O14" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O16" r:id="rId7"/>
+    <hyperlink ref="O17" r:id="rId8"/>
+    <hyperlink ref="O18" r:id="rId9"/>
+    <hyperlink ref="O20" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId11"/>

</xml_diff>